<commit_message>
35 Opp eng comments changes
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTC0036135_ValidationOfCommentsAndMappingOnConvertingOpportunityToEngagementCF.xlsx
+++ b/TestData/LV_TMTC0036135_ValidationOfCommentsAndMappingOnConvertingOpportunityToEngagementCF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98C87FF7-5E73-4C69-BA34-64B744C12A15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6354E81-19E5-40FB-A8CD-179E0B0DDBF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="2" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="93">
   <si>
     <t>James Craven</t>
   </si>
@@ -248,9 +248,6 @@
     <t>Kristian M. Whalen</t>
   </si>
   <si>
-    <t>Activism Advisory</t>
-  </si>
-  <si>
     <t>IndustryGroup/HLSector</t>
   </si>
   <si>
@@ -315,6 +312,15 @@
   </si>
   <si>
     <t>Jennie Stewart</t>
+  </si>
+  <si>
+    <t>Stage</t>
+  </si>
+  <si>
+    <t>Verbally Engaged</t>
+  </si>
+  <si>
+    <t>Buyside</t>
   </si>
 </sst>
 </file>
@@ -1033,13 +1039,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1047,7 +1053,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1055,28 +1061,28 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B3" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B5" t="s">
         <v>85</v>
-      </c>
-      <c r="B5" t="s">
-        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -1087,17 +1093,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0293C6CF-D2AF-4FB5-B989-23A4E6860FD2}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1110,24 +1116,24 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D296AE2-31EA-40C7-99FB-9B7E70535054}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1139,15 +1145,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFD13242-055E-41A8-80D8-6F50F1B57F7C}">
   <dimension ref="A1:AE2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
@@ -1158,7 +1164,7 @@
         <v>12</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>13</v>
@@ -1238,19 +1244,22 @@
       <c r="AD1" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
+      <c r="AE1" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>39</v>
       </c>
       <c r="B2" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>68</v>
+      <c r="C2" t="s">
+        <v>92</v>
       </c>
       <c r="D2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E2" t="s">
         <v>40</v>
@@ -1330,8 +1339,8 @@
       <c r="AD2" t="s">
         <v>55</v>
       </c>
-      <c r="AE2">
-        <v>10</v>
+      <c r="AE2" t="s">
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -1344,19 +1353,19 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F2CDCD2-7F5E-40FD-BAB3-4BCEC31CD21E}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>56</v>
       </c>
@@ -1382,7 +1391,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>50</v>
       </c>
@@ -1416,66 +1425,66 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9447574-C5CB-49C4-BC94-993C1D07E71B}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="60.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="60.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>74</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B2" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>76</v>
       </c>
-      <c r="C2" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>77</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>78</v>
       </c>
-      <c r="C3" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
         <v>79</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>80</v>
       </c>
-      <c r="C4" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
         <v>81</v>
       </c>
-      <c r="B5" t="s">
-        <v>82</v>
-      </c>
       <c r="C5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -1486,19 +1495,19 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D9F45E-433C-43E3-9F2A-8F8E09891021}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="59.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="59.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>83</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
360135 CAO change June 4 2025
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTC0036135_ValidationOfCommentsAndMappingOnConvertingOpportunityToEngagementCF.xlsx
+++ b/TestData/LV_TMTC0036135_ValidationOfCommentsAndMappingOnConvertingOpportunityToEngagementCF.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6354E81-19E5-40FB-A8CD-179E0B0DDBF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A7843F5-59B6-4D91-AB5E-038BF2A1E7CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1039,13 +1039,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1053,7 +1053,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1061,7 +1061,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>86</v>
       </c>
@@ -1069,7 +1069,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>89</v>
       </c>
@@ -1077,7 +1077,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>84</v>
       </c>
@@ -1093,17 +1093,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0293C6CF-D2AF-4FB5-B989-23A4E6860FD2}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1116,22 +1116,22 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D296AE2-31EA-40C7-99FB-9B7E70535054}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>70</v>
       </c>
@@ -1145,15 +1145,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFD13242-055E-41A8-80D8-6F50F1B57F7C}">
   <dimension ref="A1:AE2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
@@ -1248,7 +1248,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>39</v>
       </c>
@@ -1353,19 +1353,19 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F2CDCD2-7F5E-40FD-BAB3-4BCEC31CD21E}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>56</v>
       </c>
@@ -1391,7 +1391,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>50</v>
       </c>
@@ -1425,14 +1425,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9447574-C5CB-49C4-BC94-993C1D07E71B}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="60.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="60.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>72</v>
       </c>
@@ -1443,7 +1443,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>74</v>
       </c>
@@ -1454,7 +1454,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>76</v>
       </c>
@@ -1465,7 +1465,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>78</v>
       </c>
@@ -1476,7 +1476,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>80</v>
       </c>
@@ -1495,17 +1495,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D9F45E-433C-43E3-9F2A-8F8E09891021}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="59.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="59.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>83</v>
       </c>

</xml_diff>

<commit_message>
Juny 25 changes 2
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTC0036135_ValidationOfCommentsAndMappingOnConvertingOpportunityToEngagementCF.xlsx
+++ b/TestData/LV_TMTC0036135_ValidationOfCommentsAndMappingOnConvertingOpportunityToEngagementCF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A7843F5-59B6-4D91-AB5E-038BF2A1E7CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BA634D8-85ED-4F6E-B9D0-C6EC665E1F2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="708" windowWidth="23256" windowHeight="12456" tabRatio="548" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="2" r:id="rId1"/>
@@ -1039,13 +1039,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1053,7 +1053,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1061,7 +1061,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>86</v>
       </c>
@@ -1069,7 +1069,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>89</v>
       </c>
@@ -1077,7 +1077,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>84</v>
       </c>
@@ -1093,17 +1093,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0293C6CF-D2AF-4FB5-B989-23A4E6860FD2}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1116,22 +1116,22 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D296AE2-31EA-40C7-99FB-9B7E70535054}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>70</v>
       </c>
@@ -1145,15 +1145,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFD13242-055E-41A8-80D8-6F50F1B57F7C}">
   <dimension ref="A1:AE2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.140625" customWidth="1"/>
+    <col min="28" max="28" width="4.28515625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="16.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
@@ -1248,7 +1250,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>39</v>
       </c>
@@ -1353,19 +1355,19 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F2CDCD2-7F5E-40FD-BAB3-4BCEC31CD21E}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>56</v>
       </c>
@@ -1391,7 +1393,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>50</v>
       </c>
@@ -1425,14 +1427,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9447574-C5CB-49C4-BC94-993C1D07E71B}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="60.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="60.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>72</v>
       </c>
@@ -1443,7 +1445,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>74</v>
       </c>
@@ -1454,7 +1456,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>76</v>
       </c>
@@ -1465,7 +1467,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>78</v>
       </c>
@@ -1476,7 +1478,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>80</v>
       </c>
@@ -1495,17 +1497,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D9F45E-433C-43E3-9F2A-8F8E09891021}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="59.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="59.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>83</v>
       </c>

</xml_diff>